<commit_message>
Update code with latest changes
</commit_message>
<xml_diff>
--- a/public/Combined-Input.xlsx
+++ b/public/Combined-Input.xlsx
@@ -9520,8 +9520,10 @@
       <c r="K87" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L87" t="n">
-        <v>2128</v>
+      <c r="L87" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M87" t="inlineStr">
         <is>
@@ -9623,8 +9625,10 @@
       <c r="K88" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L88" t="n">
-        <v>1828</v>
+      <c r="L88" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M88" t="inlineStr">
         <is>
@@ -9726,8 +9730,10 @@
       <c r="K89" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L89" t="n">
-        <v>1828</v>
+      <c r="L89" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M89" t="inlineStr">
         <is>
@@ -9829,8 +9835,10 @@
       <c r="K90" t="n">
         <v>1000471622</v>
       </c>
-      <c r="L90" t="n">
-        <v>1764</v>
+      <c r="L90" t="inlineStr">
+        <is>
+          <t>Verizon-Verizon Flex - H&amp;M -VZ</t>
+        </is>
       </c>
       <c r="M90" t="inlineStr">
         <is>
@@ -9932,8 +9940,10 @@
       <c r="K91" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L91" t="n">
-        <v>2278</v>
+      <c r="L91" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M91" t="inlineStr">
         <is>
@@ -10035,8 +10045,10 @@
       <c r="K92" t="n">
         <v>1000471622</v>
       </c>
-      <c r="L92" t="n">
-        <v>1764</v>
+      <c r="L92" t="inlineStr">
+        <is>
+          <t>Verizon-Verizon Flex - H&amp;M -VZ</t>
+        </is>
       </c>
       <c r="M92" t="inlineStr">
         <is>
@@ -10136,8 +10148,8 @@
       <c r="K93" t="e">
         <v>#N/A</v>
       </c>
-      <c r="L93" t="n">
-        <v>1828</v>
+      <c r="L93" t="e">
+        <v>#N/A</v>
       </c>
       <c r="M93" t="e">
         <v>#N/A</v>
@@ -10237,8 +10249,10 @@
       <c r="K94" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L94" t="n">
-        <v>2360</v>
+      <c r="L94" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M94" t="inlineStr">
         <is>
@@ -10340,8 +10354,10 @@
       <c r="K95" t="n">
         <v>1000471622</v>
       </c>
-      <c r="L95" t="n">
-        <v>2054</v>
+      <c r="L95" t="inlineStr">
+        <is>
+          <t>Verizon-Verizon Flex - H&amp;M -VZ</t>
+        </is>
       </c>
       <c r="M95" t="inlineStr">
         <is>
@@ -10443,8 +10459,10 @@
       <c r="K96" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L96" t="n">
-        <v>2054</v>
+      <c r="L96" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M96" t="inlineStr">
         <is>
@@ -10546,8 +10564,10 @@
       <c r="K97" t="n">
         <v>1000471622</v>
       </c>
-      <c r="L97" t="n">
-        <v>2054</v>
+      <c r="L97" t="inlineStr">
+        <is>
+          <t>Verizon-Verizon Flex - H&amp;M -VZ</t>
+        </is>
       </c>
       <c r="M97" t="inlineStr">
         <is>
@@ -10649,8 +10669,10 @@
       <c r="K98" t="n">
         <v>1000471622</v>
       </c>
-      <c r="L98" t="n">
-        <v>1888</v>
+      <c r="L98" t="inlineStr">
+        <is>
+          <t>Verizon-Verizon Flex - H&amp;M -VZ</t>
+        </is>
       </c>
       <c r="M98" t="inlineStr">
         <is>
@@ -10752,8 +10774,10 @@
       <c r="K99" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L99" t="n">
-        <v>1828</v>
+      <c r="L99" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M99" t="inlineStr">
         <is>
@@ -10855,8 +10879,10 @@
       <c r="K100" t="n">
         <v>1000471622</v>
       </c>
-      <c r="L100" t="n">
-        <v>1888</v>
+      <c r="L100" t="inlineStr">
+        <is>
+          <t>Verizon-Verizon Flex - H&amp;M -VZ</t>
+        </is>
       </c>
       <c r="M100" t="inlineStr">
         <is>
@@ -10958,8 +10984,10 @@
       <c r="K101" t="n">
         <v>1000471622</v>
       </c>
-      <c r="L101" t="n">
-        <v>1656</v>
+      <c r="L101" t="inlineStr">
+        <is>
+          <t>Verizon-Verizon Flex - H&amp;M -VZ</t>
+        </is>
       </c>
       <c r="M101" t="inlineStr">
         <is>
@@ -11061,8 +11089,10 @@
       <c r="K102" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L102" t="n">
-        <v>2128</v>
+      <c r="L102" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M102" t="inlineStr">
         <is>
@@ -11164,8 +11194,10 @@
       <c r="K103" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L103" t="n">
-        <v>2054</v>
+      <c r="L103" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M103" t="inlineStr">
         <is>
@@ -11267,8 +11299,10 @@
       <c r="K104" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L104" t="n">
-        <v>2054</v>
+      <c r="L104" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M104" t="inlineStr">
         <is>
@@ -11370,8 +11404,10 @@
       <c r="K105" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L105" t="n">
-        <v>1764</v>
+      <c r="L105" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M105" t="inlineStr">
         <is>
@@ -11473,8 +11509,10 @@
       <c r="K106" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L106" t="n">
-        <v>2128</v>
+      <c r="L106" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M106" t="inlineStr">
         <is>
@@ -11576,8 +11614,10 @@
       <c r="K107" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L107" t="n">
-        <v>1764</v>
+      <c r="L107" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M107" t="inlineStr">
         <is>
@@ -11679,8 +11719,10 @@
       <c r="K108" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L108" t="n">
-        <v>2128</v>
+      <c r="L108" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M108" t="inlineStr">
         <is>
@@ -11782,8 +11824,10 @@
       <c r="K109" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L109" t="n">
-        <v>2857</v>
+      <c r="L109" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M109" t="inlineStr">
         <is>
@@ -11885,8 +11929,10 @@
       <c r="K110" t="n">
         <v>1000471622</v>
       </c>
-      <c r="L110" t="n">
-        <v>1764</v>
+      <c r="L110" t="inlineStr">
+        <is>
+          <t>Verizon-Verizon Flex - H&amp;M -VZ</t>
+        </is>
       </c>
       <c r="M110" t="inlineStr">
         <is>
@@ -11988,8 +12034,10 @@
       <c r="K111" t="n">
         <v>1000471622</v>
       </c>
-      <c r="L111" t="n">
-        <v>1764</v>
+      <c r="L111" t="inlineStr">
+        <is>
+          <t>Verizon-Verizon Flex - H&amp;M -VZ</t>
+        </is>
       </c>
       <c r="M111" t="inlineStr">
         <is>
@@ -12091,8 +12139,10 @@
       <c r="K112" t="n">
         <v>1000471622</v>
       </c>
-      <c r="L112" t="n">
-        <v>1764</v>
+      <c r="L112" t="inlineStr">
+        <is>
+          <t>Verizon-Verizon Flex - H&amp;M -VZ</t>
+        </is>
       </c>
       <c r="M112" t="inlineStr">
         <is>
@@ -12194,8 +12244,10 @@
       <c r="K113" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L113" t="n">
-        <v>2054</v>
+      <c r="L113" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M113" t="inlineStr">
         <is>
@@ -12297,8 +12349,10 @@
       <c r="K114" t="n">
         <v>1000458633</v>
       </c>
-      <c r="L114" t="n">
-        <v>2857</v>
+      <c r="L114" t="inlineStr">
+        <is>
+          <t>VDSI-Flex-H&amp;M-Base Marketing</t>
+        </is>
       </c>
       <c r="M114" t="inlineStr">
         <is>

</xml_diff>